<commit_message>
Complete documentation and update sample roster
</commit_message>
<xml_diff>
--- a/Fake_Random_Names.xlsx
+++ b/Fake_Random_Names.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\918839355\Desktop\412\Attendance App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0D6E7B-8726-4776-8DD9-5401D35AE83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{925B21A5-B546-4FCB-B5C0-AB77EE6AFD9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -176,14 +176,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -235,20 +228,20 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6"/>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -468,7 +461,7 @@
     <col min="2" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="14.3">
+    <row r="1" spans="1:2" ht="14.3" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>